<commit_message>
data: re-ingest Week 21 other-channels sales (all 4 brands updated)
  • other_channels.xlsx replaced for Audio Array / Nexlev / Tonor /
    White Mulberry
  • Regenerated weekly_sales_snapshot

Returns + other snapshots unchanged after rerun (no impact downstream).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 21/Audio_Array/other_channels.xlsx
+++ b/data/raw/sales/Week 21/Audio_Array/other_channels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 21\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB41CC96-CA35-40F4-A2E7-CF4BF0CC086A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC768DA0-060B-41EF-9215-127BBA035159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2227,7 +2227,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:W915"/>
+  <dimension ref="A1:V915"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" customWidth="1"/>
@@ -2236,10 +2236,10 @@
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="19.88671875" customWidth="1"/>
     <col min="6" max="6" width="11.6640625" customWidth="1"/>
-    <col min="7" max="23" width="8.6640625" customWidth="1"/>
+    <col min="7" max="22" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
         <v>5</v>
       </c>
@@ -2274,9 +2274,8 @@
       <c r="T1" s="4"/>
       <c r="U1" s="4"/>
       <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-    </row>
-    <row r="2" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
         <v>12</v>
       </c>
@@ -2293,10 +2292,10 @@
         <v>8</v>
       </c>
       <c r="F2" s="16">
-        <v>40792</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>34569</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
         <v>12</v>
       </c>
@@ -2313,10 +2312,10 @@
         <v>14</v>
       </c>
       <c r="F3" s="16">
-        <v>31486</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>26683</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
         <v>12</v>
       </c>
@@ -2333,10 +2332,10 @@
         <v>6</v>
       </c>
       <c r="F4" s="16">
-        <v>16194</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13724</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>12</v>
       </c>
@@ -2356,7 +2355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
         <v>12</v>
       </c>
@@ -2373,10 +2372,10 @@
         <v>3</v>
       </c>
       <c r="F6" s="16">
-        <v>10585</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>8970</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
         <v>12</v>
       </c>
@@ -2393,10 +2392,10 @@
         <v>3</v>
       </c>
       <c r="F7" s="16">
-        <v>5697</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>4828</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
         <v>12</v>
       </c>
@@ -2416,7 +2415,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
         <v>12</v>
       </c>
@@ -2433,10 +2432,10 @@
         <v>5</v>
       </c>
       <c r="F9" s="16">
-        <v>6295</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>5335</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
         <v>12</v>
       </c>
@@ -2453,15 +2452,15 @@
         <v>1</v>
       </c>
       <c r="F10" s="16">
-        <v>1999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:23" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:22" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>